<commit_message>
july 30 2025 update
</commit_message>
<xml_diff>
--- a/data/package_table.xlsx
+++ b/data/package_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c5c54cfb0e9536a4/Ongoing Work/Teaching/Leiden/Statistics II (R Version)/R Files/R Overviews/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jar68\Documents\github\statistics2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{5CDBA9C0-EE4D-46E0-890A-6CD0963DF9B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BE7F874-9FB3-49CA-8BEB-ED3004C54625}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9FA79C-41BB-4508-89D9-CD1B81371939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2B8B4975-3241-4F90-AA0B-8056DD3AD8F2}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B8B4975-3241-4F90-AA0B-8056DD3AD8F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
   <si>
     <t>Package</t>
   </si>
@@ -255,6 +255,15 @@
   </si>
   <si>
     <t>slopes() &amp; avg_slopes()</t>
+  </si>
+  <si>
+    <t>fastDummies</t>
+  </si>
+  <si>
+    <t>dummy_cols()</t>
+  </si>
+  <si>
+    <t>Creating dummy variables for categorical variables</t>
   </si>
 </sst>
 </file>
@@ -319,9 +328,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -359,7 +368,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -465,7 +474,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -607,7 +616,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -615,16 +624,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF3BFA38-E02F-493B-B51E-E2406CAE5CC4}">
-  <dimension ref="A1:D28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -638,7 +647,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -652,7 +661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -666,7 +675,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -680,7 +689,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -694,7 +703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -708,7 +717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -722,7 +731,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -736,7 +745,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -750,7 +759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -764,7 +773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -778,7 +787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>48</v>
       </c>
@@ -792,7 +801,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -806,7 +815,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>48</v>
       </c>
@@ -820,7 +829,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -834,7 +843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -848,7 +857,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>66</v>
       </c>
@@ -862,7 +871,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -876,7 +885,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -890,7 +899,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -904,7 +913,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -918,7 +927,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -932,7 +941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -946,7 +955,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>59</v>
       </c>
@@ -960,7 +969,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -974,7 +983,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>22</v>
       </c>
@@ -988,7 +997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>22</v>
       </c>
@@ -1002,7 +1011,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1014,6 +1023,20 @@
       </c>
       <c r="D28">
         <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>